<commit_message>
chore(tm): record archive snapshot 快照-0001 with checksum and evidence-0007
git archive of 8a5c71d -> 协作/归档/dcg-tm-v3.4.zip (197 files, SHA256 f93cc611...), restore verification passed; 27-归档快照与校验 carries the verifiable record, 26-归档清单 registers the snapshot and the two new evidence docs.
</commit_message>
<xml_diff>
--- a/协作/26-归档清单.xlsx
+++ b/协作/26-归档清单.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K70"/>
+  <dimension ref="A1:K74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4323,6 +4323,214 @@
       <c r="K70" t="inlineStr">
         <is>
           <t>登记后随规范升版重建</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>归档-0070</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>27-归档快照与校验.xlsx</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>记录</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>v3.4</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>集成发布</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>G8</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>证据-0007</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>在档</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>归档-0071</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>24-证据/证据-0006.docx</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>证据</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>测试验证</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>G6</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>证据-0006</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>在档</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>归档-0072</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>24-证据/证据-0007.docx</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>证据</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>测试验证</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>G6</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>证据-0007</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>长期</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>在档</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>归档-0073</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>归档包</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>归档/dcg-tm-v3.4.zip</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>归档包</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>v3.4</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>集成发布</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>G8</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>证据-0007</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>由 提交号 8a5c71d 的 git archive 生成，197 份文件 / 1741944 字节；快照记录本身（27）不在包内，属自引用限制</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>在档</t>
         </is>
       </c>
     </row>

</xml_diff>